<commit_message>
Add architecture diagrams, concrete time-saved metrics, explicit roadmap example
- docs/architecture.md: mermaid diagrams for the whole flow, a daily run as a
  sequence, how a signal is scored, why the merge is guarded, and what makes
  runs safe to repeat. GitHub renders these, so there are no images to keep in sync.
- README: the ASCII sketch becomes a real diagram; adds what the example week
  actually saved and how that scales with call volume, with the assumption stated.
- knowledge/product.md becomes knowledge/roadmap.md — it always was the roadmap,
  the name now says so.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example-run/signal-matrix.xlsx
+++ b/example-run/signal-matrix.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +49,30 @@
       <b val="1"/>
       <color rgb="003D5A80"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="003D5A80"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004C8577"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008A6A2F"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +89,36 @@
         <fgColor rgb="00EDF1F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7E9E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F0EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EEF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF2DF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -80,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -94,6 +146,57 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -567,1184 +670,1248 @@
       </c>
     </row>
     <row r="4" ht="78" customHeight="1">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Act on a stop from the phone, not just see it</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Enhancement — Gap</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Prospect, Customer</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Not planned (Q3 mobile layout is view-only — ruled by Alex Kim 2026-08-02)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Acme Foods: 2, Vertex Motors: 2</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Seeing the line on a phone does not change anything by itself. The supervisors who have no workstation are the same people who have to tag the stop, acknowledge the alert and record what they did — and that still means walking to a computer, which is the reason they do not do it. Acme's pilot is scored on supervisors acting during the shift, not on them looking, and the committed Q3 mobile layout is view-only, so the acting half has no roadmap home. Caveat, stated plainly: Vertex's importance 2 is the size of the no-desk population; asked directly on the same call they said read-only was fine. Acme is the only account that has so far tied acting to a consequence — see Opportunity briefs/OB-act-from-the-phone.md.</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Acme Foods: "If my supervisors act on something during the shift, at least twice a week, without me telling them to. That is the whole test."
+Vertex Motors: "Half my supervisors do not sit at a desk. They have a phone in their pocket and that is it."</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="n"/>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>https://example.com/calls/1001
+https://example.com/calls/1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Read-only view of line status on a phone</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Roadmap validation</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Prospect, Customer</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Unclear — needs Alex Kim (Mobile layout Q3 is read-only)</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>On roadmap — committed (Mobile layout, Q3 — view-only)</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: 2, Vertex Motors: 2</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H5" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Supervisors who spend the shift on the floor have no workstation, so they never see line status while they could still act on it. They want to check the line from the phone already in their pocket; read-only is enough.</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>Supervisors who spend the shift on the floor have no workstation, so they never see line status while they could still act on it. They want to check the line from the phone already in their pocket; read-only is enough. The acting half of this need was split out on 2026-08-02, after Alex Kim ruled the Q3 layout view-only — see “Act on a stop from the phone, not just see it”.</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Vertex Motors: "Half my supervisors do not sit at a desk. They have a phone in their pocket and that is it."
 Acme Foods: "We are there on line three. Not on line one, because line one's supervisor does not sit at a computer."</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="M5" s="13" t="n"/>
+      <c r="N5" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1002
 https://example.com/calls/1005</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="78" customHeight="1">
-      <c r="A5" s="6" t="n">
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Surface recurring stop patterns automatically</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Roadmap validation</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Prospect, Customer</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>On roadmap — discovery (Root-cause suggestions)</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Acme Foods: 1, Vertex Motors: 1</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Surface recurring stop patterns automatically</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Roadmap validation</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Prospect, Customer</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>On roadmap — discovery (Root-cause suggestions)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Acme Foods: 1, Vertex Motors: 1</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="6" t="n">
+      <c r="H6" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Repeating stops are only noticed when somebody happens to scan several days of the log by eye. Users want the system to point out the pattern itself — same station, same shift, three days running — rather than only categorising stops.</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: "If the system spotted that and said it out loud, I would trust it more than any chart."
 Acme Foods: "It was seeing the same stop reason three days running. Nobody had noticed."</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L6" s="8" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="M5" s="6" t="n"/>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="M6" s="8" t="n"/>
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1002
 https://example.com/calls/1005</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Let customers edit the downtime reason-code list</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Enhancement — Gap</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Prospect, Customer</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Not planned</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: 2</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G7" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H7" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>The list of downtime reason codes is fixed and can only be changed by support, so it drifts out of date and operators dump unmatched stops into 'other'. Customers want to add, retire and group reasons themselves so downtime analysis stays usable.</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J7" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: "My CI lead still cannot edit the stop reason list. She has asked me three times."</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K7" s="13" t="inlineStr">
         <is>
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L7" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="M6" s="6" t="n"/>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="M7" s="13" t="n"/>
+      <c r="N7" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1001
 https://example.com/calls/1005</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="78" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Alerts delivered into the chat tool people use on shift</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>New feature</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Unclear — needs Alex Kim</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Lumen Devices: 2</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H8" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Alerts that arrive by email are not seen, because nobody on the floor reads email during a shift. Alerts need to land in the chat tool the shift already has open.</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Lumen Devices: "I want them in Teams, not by email. Nobody here reads email during the shift."</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L8" s="8" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="M7" s="6" t="n"/>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="M8" s="8" t="n"/>
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1004</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="78" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Bug — output double-counted after a line restart</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Shipped (Line dashboard)</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: 2</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H9" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>After a line restart the counter reported roughly double the real output for a full day. Reported as fixed on the call; logged because recurrence would matter.</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: "The numbers on line three were wrong for a full day. Output showed roughly double."</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K9" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L9" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="M8" s="6" t="n"/>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1005</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Compare a line against the same day last week</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>Enhancement — Amplify</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Prospect</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Shipped (Line dashboard)</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: 2</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H10" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>The like-for-like day comparison already in the dashboard replaces a spreadsheet the customer had been maintaining by hand for a year — worth leading with, because it removes a recurring weekly task rather than adding a new screen.</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: "That is the argument I have been trying to make with a spreadsheet for a year."</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L10" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M9" s="6" t="n"/>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="M10" s="8" t="n"/>
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1002</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Compare the same line across shifts and crews</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Roadmap validation</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>On roadmap — committed (Shift comparison view, Q2)</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Lumen Devices: 2</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G11" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H11" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I11" s="13" t="inlineStr">
         <is>
           <t>Differences between crews on the same line are invisible today, and a customer has already promised their own management a shift comparison by April.</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>Lumen Devices: "I told the plant manager we'd have them in April."</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K11" s="13" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="L11" s="13" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="M11" s="13" t="n"/>
+      <c r="N11" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1004</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Create and remove users in bulk</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Enhancement — Gap</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Unclear — needs Alex Kim</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Halden Pumps: 2</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Accounts can only be created one at a time in the admin panel, which does not scale past a couple of lines and produces typos. Admins want bulk import, or accounts that follow the company directory as people move between lines.</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>Halden Pumps: "You are asking me to create fifty-two users by hand. That is not sustainable at seven lines."</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="M12" s="8" t="n"/>
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1003</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="78" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+    <row r="13" ht="78" customHeight="1">
+      <c r="A13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Flag numbers that look implausible</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>New feature</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Not planned</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: 2</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G13" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H13" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I13" s="13" t="inlineStr">
         <is>
           <t>When a reading is wrong, nothing says so, and people act on it for a full day before anyone notices. Users want obviously implausible values flagged automatically so trust in the data survives a bad reading.</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J13" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: "A wrong number I trust is worse than no number."</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K13" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="L13" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1005</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
+    <row r="14" ht="78" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>In-product screen showing what personal data is stored</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>New feature</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Not planned</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Halden Pumps: 2</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>Employee representatives will not sign off on a policy document; they want to be shown, live in the product, exactly what is recorded about an individual operator. Without it the rollout cannot start.</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>Halden Pumps: "This is the condition the whole rollout hangs on. Everything else we can work around."</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="6" t="inlineStr">
+      <c r="M14" s="8" t="n"/>
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1003</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="78" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
+    <row r="15" ht="78" customHeight="1">
+      <c r="A15" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>One view across all plants</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Roadmap validation</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>Prospect, Customer</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>On roadmap — discovery (Multi-site rollup)</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: 1</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G15" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H15" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I15" s="13" t="inlineStr">
         <is>
           <t>Data stops at the plant boundary, so a regional manager has to open one account per site. They want every plant on a single screen.</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J15" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: "He wants all four plants on one screen."</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K15" s="13" t="inlineStr">
         <is>
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L15" s="13" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="M15" s="13" t="n"/>
+      <c r="N15" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1001
 https://example.com/calls/1005</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="78" customHeight="1">
-      <c r="A15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
+    <row r="16" ht="78" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Scheduled data feed into the customer's own warehouse</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Enhancement — Gap</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Prospect</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Deferred (Public API)</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: 2</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G16" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H16" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>Getting the numbers out means a person clicking download, so the data cannot live inside the customer's own reporting stack. They want an endpoint their systems can pull from on a schedule.</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: "We want the raw numbers in our own warehouse. Not a CSV someone downloads. An endpoint we can pull from every night."</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M15" s="6" t="n"/>
-      <c r="N15" s="6" t="inlineStr">
+      <c r="M16" s="8" t="n"/>
+      <c r="N16" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1002</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="78" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+    <row r="17" ht="78" customHeight="1">
+      <c r="A17" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Separate planned maintenance from unplanned downtime</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Enhancement — Gap</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>On roadmap — discovery (Maintenance-system integration)</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Lumen Devices: 2</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G17" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H17" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>Planned maintenance is counted as availability loss, so the availability figure looks wrong to plant leadership and the dashboard cannot be shown in management meetings. Planned stops need to be excluded or reported separately.</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>Lumen Devices: "I need that. As long as the number looks wrong, I can't show it in the factory meeting."</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="K17" s="13" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L17" s="13" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="M16" s="6" t="n"/>
-      <c r="N16" s="6" t="inlineStr">
+      <c r="M17" s="13" t="n"/>
+      <c r="N17" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1004</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="78" customHeight="1">
-      <c r="A17" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
+    <row r="18" ht="78" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Single sign-on with the corporate identity provider</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Roadmap validation</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Prospect</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>On roadmap — committed (Single sign-on / SAML, Q3)</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: 2</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="H18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Enterprise IT will not approve a tool that keeps its own local accounts. SSO through the company identity provider is a security-review gate, not a preference.</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>Vertex Motors: "I am not saying no. I am saying it is a gate, not a wish."</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L18" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M17" s="6" t="n"/>
-      <c r="N17" s="6" t="inlineStr">
+      <c r="M18" s="8" t="n"/>
+      <c r="N18" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1002</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="78" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
+    <row r="19" ht="78" customHeight="1">
+      <c r="A19" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Tell me when the line drifts, during the shift</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>Roadmap validation</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>Prospect</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>On roadmap — committed (Real-time alerts, Q2)</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: 2</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G19" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H19" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="I19" s="13" t="inlineStr">
         <is>
           <t>Shortfalls are discovered hours later from a manual count or the next morning's report, when nothing can be done about them. Users want to be told while the shift is still running.</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>Acme Foods: "That is the difference between us running a pilot and us not running a pilot."</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="K19" s="13" t="inlineStr">
         <is>
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L19" s="13" t="inlineStr">
         <is>
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="M18" s="6" t="n"/>
-      <c r="N18" s="6" t="inlineStr">
+      <c r="M19" s="13" t="n"/>
+      <c r="N19" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1001</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="78" customHeight="1">
-      <c r="A19" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
+    <row r="20" ht="78" customHeight="1">
+      <c r="A20" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Bug — line filter resets when the date range changes</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Shipped (Line dashboard)</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Halden Pumps: 1</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G20" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>Filtering the dashboard to one line and then changing the date range silently returns the view to all lines, so a user can read the wrong figures without noticing.</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>Halden Pumps: "When I filter the dashboard to a single line and then change the date range, the filter resets to all lines. Every time."</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L20" s="8" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="M20" s="8" t="n"/>
+      <c r="N20" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1003</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="78" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Choose when the weekly report is generated</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Enhancement — Gap</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="23" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>Not planned</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Halden Pumps: 1</t>
         </is>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G21" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H21" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="I21" s="13" t="inlineStr">
         <is>
           <t>The weekly report runs on a fixed schedule that does not match every plant's week, so it consistently misses the shift that opens the week. Customers want to set the day and time themselves.</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>Halden Pumps: "Our week starts Sunday night with the late shift, so the report always misses it."</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="K21" s="13" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L21" s="13" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="M20" s="6" t="n"/>
-      <c r="N20" s="6" t="inlineStr">
+      <c r="M21" s="13" t="n"/>
+      <c r="N21" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1003</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="78" customHeight="1">
-      <c r="A21" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
+    <row r="22" ht="78" customHeight="1">
+      <c r="A22" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Read planned stops from the maintenance system</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Roadmap validation</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>On roadmap — discovery (Maintenance-system integration)</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Lumen Devices: 1</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G22" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="H22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>Tagging which stops were planned is manual, even though the work orders already exist in the maintenance system. Reading them would classify those stops automatically.</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>Lumen Devices: "If you could read that, the assignment would be automatic."</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L22" s="8" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="M21" s="6" t="n"/>
-      <c r="N21" s="6" t="inlineStr">
+      <c r="M22" s="8" t="n"/>
+      <c r="N22" s="8" t="inlineStr">
         <is>
           <t>https://example.com/calls/1004</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="78" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
+    <row r="23" ht="78" customHeight="1">
+      <c r="A23" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Weekly report stays legible when printed large</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Enhancement — Gap</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>Not planned</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Lumen Devices: 1</t>
         </is>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G23" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H23" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I23" s="13" t="inlineStr">
         <is>
           <t>The weekly PDF is printed and pinned to a notice board, but the layout does not scale up, so the type is too small to read from standing distance.</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J23" s="13" t="inlineStr">
         <is>
           <t>Lumen Devices: "The font is too small when printed on A3. Not a big deal."</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="K23" s="13" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="L23" s="13" t="inlineStr">
         <is>
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="M22" s="6" t="n"/>
-      <c r="N22" s="6" t="inlineStr">
+      <c r="M23" s="13" t="n"/>
+      <c r="N23" s="13" t="inlineStr">
         <is>
           <t>https://example.com/calls/1004</t>
         </is>
@@ -2134,7 +2301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2291,6 +2458,55 @@
         <v>5</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>week</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>19</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>47%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Measure time saved from real call length, and apply the brand palette and type
Time saved was an assumption (calls x 15 min). It is now the summed real duration of
the calls the system read, recorded per call in the ledger; only calls whose length was
never captured fall back to the estimate, and reports say how many. Metrics also project
forward from the observed rate: at 5 calls a week the example reaches 61 h by 31 Dec.

Also: the rate is measured over the period the calls actually span, so backfilling one
busy week no longer reads as a slow year.

Visual identity: dusty blue, matcha and ballet pink replace the placeholder palette, with
serif headlines, sans body and mono stamps — all falling back to fonts every machine has,
so PDFs render identically anywhere. All three example documents re-rendered.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example-run/signal-matrix.xlsx
+++ b/example-run/signal-matrix.xlsx
@@ -2073,7 +2073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2082,6 +2082,7 @@
     <col width="54" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2129,6 +2130,11 @@
           <t>Call type</t>
         </is>
       </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Duration (min)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2161,6 +2167,9 @@
           <t>Prospect</t>
         </is>
       </c>
+      <c r="G4" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2193,6 +2202,9 @@
           <t>Prospect</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2225,6 +2237,9 @@
           <t>Implementation</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2257,6 +2272,9 @@
           <t>Customer</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2288,6 +2306,9 @@
         <is>
           <t>Customer</t>
         </is>
+      </c>
+      <c r="G8" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>